<commit_message>
Apply author decisions: WSA in g/g (>0.053 mm), green manure supplementary for CA, serials from 164
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyYAcBGZJWQtif7Vn7og8L
</commit_message>
<xml_diff>
--- a/META_ANALYSIS_NEW_updated_01.xlsx
+++ b/META_ANALYSIS_NEW_updated_01.xlsx
@@ -1174,7 +1174,7 @@
       </c>
       <c r="B2" s="41" t="inlineStr">
         <is>
-          <t>Started 2026-10-05. All data rows of the old master were removed at the author's request; serials start at 1. The history entries further down describe the OLD master (updated 53) and are kept only as the rulebook.</t>
+          <t>Started 2026-10-05. All data rows of the old master were removed at the author's request; serials continue from the old master, starting at 164, so the two files can be merged. The history entries further down describe the OLD master (updated 53) and are kept only as the rulebook.</t>
         </is>
       </c>
     </row>
@@ -23315,7 +23315,7 @@
     <row r="2" ht="15" customHeight="1">
       <c r="BA2" s="23" t="inlineStr">
         <is>
-          <t>% water-stable aggregates</t>
+          <t>g/g soil (water-stable aggregates = sum of ALL water-stable fractions &gt; 0.053 mm; % / 100)</t>
         </is>
       </c>
     </row>
@@ -25479,7 +25479,7 @@
       </c>
       <c r="C80" s="49" t="inlineStr">
         <is>
-          <t>NEW workbook: built on the updated 53 structure with NO previous data carried over. Serial numbers start at 1. Each upload is saved as a new numbered version (META_ANALYSIS_NEW_updated_NN.xlsx).</t>
+          <t>NEW workbook: built on the updated 53 structure with NO previous data carried over. Serial numbers CONTINUE from the old master: the first new study is 164 (old master ends at 163), so the two files can be merged. Each upload is saved as a new numbered version (META_ANALYSIS_NEW_updated_NN.xlsx).</t>
         </is>
       </c>
       <c r="D80" s="49" t="inlineStr">
@@ -25514,7 +25514,7 @@
       </c>
       <c r="D81" s="49" t="inlineStr">
         <is>
-          <t>Every parameter sheet carries &lt;prefix&gt;pCA, pZT, pMT, pMTR right after &lt;prefix&gt;DTR (olive-green headers). These treatments are NO LONGER excluded under the rotation-matching rule (rule 22) and are NOT entered in the CA / ZT / MT / MTR columns; they go to the p-columns. The reverse mismatch (ZT / no-till rice + conventional wheat, RNT-WCT) stays EXCLUDED. MT vs MTR for the wheat phase follows the rotary rule (rule 13).</t>
+          <t>Every parameter sheet carries &lt;prefix&gt;pCA, pZT, pMT, pMTR right after &lt;prefix&gt;DTR (olive-green headers). These treatments are NO LONGER excluded under the rotation-matching rule (rule 22) and are NOT entered in the CA / ZT / MT / MTR columns; they go to the p-columns. The reverse mismatch (ZT / no-till rice + conventional wheat, RNT-WCT) stays EXCLUDED (author re-confirmed). MT vs MTR for the wheat phase follows the rotary rule (rule 13).</t>
         </is>
       </c>
       <c r="E81" s="49" t="inlineStr">
@@ -25599,12 +25599,12 @@
       </c>
       <c r="C84" s="49" t="inlineStr">
         <is>
-          <t>Third crop / green manure (mungbean, Sesbania, etc.) in a rice-wheat system: study included; green manuring counts as part of CA (supports CA).</t>
+          <t>Green manuring / a third crop (mungbean, Sesbania, etc.) in a rice-wheat system: study included. Green manuring is a SUPPLEMENTARY condition for CA, NOT a necessary one: ZT + residue = CA with or without green manure.</t>
         </is>
       </c>
       <c r="D84" s="49" t="inlineStr">
         <is>
-          <t>Flag the row 'GREEN MANURE / 3rd CROP' in Notes. If the green manure / third crop is present only in the CA treatments, the row is entered flagged so it can be dropped in a sensitivity analysis.</t>
+          <t>A green manure / third crop grown only in the CA treatment does not exclude that treatment and does not change its code; the crop is named in Notes and 'Fertilizer dose &amp; other management' ('GREEN MANURE'). Green manure never turns a non-CA treatment into CA (e.g. ZT without residue + green manure stays ZT).</t>
         </is>
       </c>
       <c r="E84" s="49" t="inlineStr">
@@ -25689,12 +25689,12 @@
       </c>
       <c r="C87" s="49" t="inlineStr">
         <is>
-          <t>WSA: when the paper gives no WSA but gives water-stable aggregate fractions, WSA = sum of the water-stable macro + micro (meso) aggregate fractions (DERIVED, flagged).</t>
+          <t>WSA = sum of ALL water-stable aggregate fractions &gt; 0.053 mm, in g/g of soil (0-1). A printed WSA in % is divided by 100; when the paper gives only the fractions, WSA is their sum (DERIVED, flagged).</t>
         </is>
       </c>
       <c r="D87" s="49" t="inlineStr">
         <is>
-          <t>Live formula referencing MACRO / MICRO rows where possible.</t>
+          <t>The silt + clay fraction (&lt; 0.053 mm) is never included. The old master (updated 53) holds WSA in % - divide by 100 when merging.</t>
         </is>
       </c>
       <c r="E87" s="49" t="inlineStr">
@@ -44807,7 +44807,7 @@
       </c>
       <c r="C13" s="76" t="inlineStr">
         <is>
-          <t>% water-stable aggregates</t>
+          <t>g/g soil (water-stable aggregates = sum of ALL water-stable fractions &gt; 0.053 mm; % / 100)</t>
         </is>
       </c>
       <c r="D13" s="76" t="n">

</xml_diff>